<commit_message>
Set August report total to actual payout 233.08 USD
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012c5okHokQRbqvr7ymitv3U
</commit_message>
<xml_diff>
--- a/financial_report_august.xlsx
+++ b/financial_report_august.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,11 @@
     </font>
     <font>
       <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -96,8 +101,8 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -931,27 +936,48 @@
         <f>SUM(B4:B12)</f>
         <v/>
       </c>
-      <c r="J14" s="8">
+      <c r="J14" s="8" t="n">
+        <v>233.08</v>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Переведено на счет: REVOLUT BANK UAB-****8045</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Расчет по курсам</t>
+        </is>
+      </c>
+      <c r="J16" s="4">
         <f>SUM(J4:J12)</f>
         <v/>
       </c>
-      <c r="K14" s="7" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>Переведено на счет: REVOLUT BANK UAB-****8045</t>
-        </is>
-      </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Синим — курсы валют (вводные). Взяты из июльского отчета Apple; курс AUD (желтый) — оценочный. Замените на курсы из раздела «Платежи и финансовые отчеты» за август.</t>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Курсовая разница</t>
+        </is>
+      </c>
+      <c r="J17" s="4">
+        <f>J14-J16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Итого 233,08 USD — фактическая сумма перевода Apple. Поступления по странам рассчитаны по курсам июльского отчета (курс AUD, желтый, — оценочный); разница с фактом показана как курсовая разница.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use Apple's August exchange rates in report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012c5okHokQRbqvr7ymitv3U
</commit_message>
<xml_diff>
--- a/financial_report_august.xlsx
+++ b/financial_report_august.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,18 +44,8 @@
     <font>
       <name val="Arial"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000000FF"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -65,11 +55,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -98,11 +83,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -578,7 +561,7 @@
         <v/>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.64</v>
+        <v>0.6953</v>
       </c>
       <c r="J4" s="4">
         <f>ROUND(H4*I4,2)</f>
@@ -619,8 +602,8 @@
         <f>D5+E5+F5-G5</f>
         <v/>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>0.7192</v>
+      <c r="I5" s="5" t="n">
+        <v>0.70199</v>
       </c>
       <c r="J5" s="4">
         <f>ROUND(H5*I5,2)</f>
@@ -661,8 +644,8 @@
         <f>D6+E6+F6-G6</f>
         <v/>
       </c>
-      <c r="I6" s="6" t="n">
-        <v>1.2338</v>
+      <c r="I6" s="5" t="n">
+        <v>1.19444</v>
       </c>
       <c r="J6" s="4">
         <f>ROUND(H6*I6,2)</f>
@@ -703,8 +686,8 @@
         <f>D7+E7+F7-G7</f>
         <v/>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>1.15598</v>
+      <c r="I7" s="5" t="n">
+        <v>1.13051</v>
       </c>
       <c r="J7" s="4">
         <f>ROUND(H7*I7,2)</f>
@@ -745,8 +728,8 @@
         <f>D8+E8+F8-G8</f>
         <v/>
       </c>
-      <c r="I8" s="6" t="n">
-        <v>1.35095</v>
+      <c r="I8" s="5" t="n">
+        <v>1.31861</v>
       </c>
       <c r="J8" s="4">
         <f>ROUND(H8*I8,2)</f>
@@ -787,8 +770,8 @@
         <f>D9+E9+F9-G9</f>
         <v/>
       </c>
-      <c r="I9" s="6" t="n">
-        <v>0.10695</v>
+      <c r="I9" s="5" t="n">
+        <v>0.10388</v>
       </c>
       <c r="J9" s="4">
         <f>ROUND(H9*I9,2)</f>
@@ -829,8 +812,8 @@
         <f>D10+E10+F10-G10</f>
         <v/>
       </c>
-      <c r="I10" s="6" t="n">
-        <v>0.58917</v>
+      <c r="I10" s="5" t="n">
+        <v>0.56369</v>
       </c>
       <c r="J10" s="4">
         <f>ROUND(H10*I10,2)</f>
@@ -871,8 +854,8 @@
         <f>D11+E11+F11-G11</f>
         <v/>
       </c>
-      <c r="I11" s="6" t="n">
-        <v>0.02072</v>
+      <c r="I11" s="5" t="n">
+        <v>0.02027</v>
       </c>
       <c r="J11" s="4">
         <f>ROUND(H11*I11,2)</f>
@@ -913,7 +896,7 @@
         <f>D12+E12+F12-G12</f>
         <v/>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="I12" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J12" s="4">
@@ -927,19 +910,20 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="6">
         <f>SUM(B4:B12)</f>
         <v/>
       </c>
-      <c r="J14" s="8" t="n">
-        <v>233.08</v>
-      </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="J14" s="7">
+        <f>SUM(J4:J12)</f>
+        <v/>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -949,35 +933,6 @@
       <c r="K15" s="3" t="inlineStr">
         <is>
           <t>Переведено на счет: REVOLUT BANK UAB-****8045</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Расчет по курсам</t>
-        </is>
-      </c>
-      <c r="J16" s="4">
-        <f>SUM(J4:J12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Курсовая разница</t>
-        </is>
-      </c>
-      <c r="J17" s="4">
-        <f>J14-J16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Итого 233,08 USD — фактическая сумма перевода Apple. Поступления по странам рассчитаны по курсам июльского отчета (курс AUD, желтый, — оценочный); разница с фактом показана как курсовая разница.</t>
         </is>
       </c>
     </row>
@@ -1016,92 +971,92 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Transaction Date</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Settlement Date</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Apple Identifier</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Developer Name</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Product Type Identifier</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Country of Sale</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Partner Share</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Extended Partner Share</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Partner Share Currency</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>Customer Price</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Customer Currency</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Sale or Return</t>
         </is>
       </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>Promo Code</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>Order Type</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>Region</t>
         </is>

</xml_diff>